<commit_message>
Amazon Clone next change
</commit_message>
<xml_diff>
--- a/Attendance.xlsx
+++ b/Attendance.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="168">
   <si>
     <t>Sr. No</t>
   </si>
@@ -535,13 +535,16 @@
   </si>
   <si>
     <t>Sanket Kunde</t>
+  </si>
+  <si>
+    <t>AA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -596,6 +599,25 @@
       <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -792,7 +814,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -804,9 +826,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -834,19 +853,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -868,6 +874,37 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1185,11 +1222,15 @@
   <dimension ref="A1:L80"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.1796875" customWidth="1"/>
+    <col min="3" max="3" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33.36328125" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" style="14" customWidth="1"/>
-    <col min="7" max="7" width="12.6328125" style="29" customWidth="1"/>
-    <col min="8" max="8" width="10.08984375" style="32" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="1.81640625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="4.26953125" style="23" customWidth="1"/>
+    <col min="8" max="8" width="3.6328125" style="26" customWidth="1"/>
+    <col min="9" max="9" width="1.90625" customWidth="1"/>
+    <col min="10" max="10" width="10.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31" thickBot="1" x14ac:dyDescent="0.4">
@@ -1205,50 +1246,56 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="24">
+      <c r="F1" s="18">
         <v>46042</v>
       </c>
-      <c r="G1" s="27">
+      <c r="G1" s="21">
         <v>46043</v>
       </c>
-      <c r="H1" s="25">
+      <c r="H1" s="19">
         <v>46044</v>
       </c>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2">
+      <c r="I1" s="18">
+        <v>46045</v>
+      </c>
+      <c r="J1" s="18">
+        <v>46049</v>
+      </c>
+      <c r="K1" s="13"/>
+    </row>
+    <row r="2" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="27">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="28">
         <v>7709797922</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H2" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
+      <c r="E2" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G2" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H2" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K2" s="30"/>
     </row>
     <row r="3" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
@@ -1263,13 +1310,13 @@
       <c r="D3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="26"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
+      <c r="E3" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="20"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
     </row>
     <row r="4" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
@@ -1284,13 +1331,13 @@
       <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="26"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
+      <c r="E4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="20"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
     </row>
     <row r="5" spans="1:11" ht="41.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
@@ -1305,13 +1352,13 @@
       <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="26"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
+      <c r="E5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="20"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
     </row>
     <row r="6" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
@@ -1326,15 +1373,15 @@
       <c r="D6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
+      <c r="E6" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
     </row>
     <row r="7" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
@@ -1349,14 +1396,14 @@
       <c r="D7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="28"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
+      <c r="E7" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="22"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
     </row>
     <row r="8" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
@@ -1371,13 +1418,13 @@
       <c r="D8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H8" s="26"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
+      <c r="E8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" s="20"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
     </row>
     <row r="9" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
@@ -1392,44 +1439,48 @@
       <c r="D9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H9" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
-    </row>
-    <row r="10" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2">
+      <c r="E9" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+    </row>
+    <row r="10" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="27">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="28">
         <v>9503424123</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G10" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H10" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
+      <c r="E10" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H10" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I10" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J10" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K10" s="30"/>
     </row>
     <row r="11" spans="1:11" ht="28" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
@@ -1444,13 +1495,13 @@
       <c r="D11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H11" s="26"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
+      <c r="E11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
     </row>
     <row r="12" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
@@ -1465,42 +1516,46 @@
       <c r="D12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H12" s="26"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-    </row>
-    <row r="13" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2">
+      <c r="E12" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="20"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+    </row>
+    <row r="13" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="27">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="28">
         <v>9112924669</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G13" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H13" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="14"/>
+      <c r="E13" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G13" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H13" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I13" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="J13" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K13" s="30"/>
     </row>
     <row r="14" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
@@ -1515,18 +1570,20 @@
       <c r="D14" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="G14" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H14" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
+      <c r="E14" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K14" s="13"/>
     </row>
     <row r="15" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
@@ -1541,13 +1598,15 @@
       <c r="D15" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="H15" s="26"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K15" s="13"/>
     </row>
     <row r="16" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
@@ -1562,14 +1621,14 @@
       <c r="D16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" s="28"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
+      <c r="E16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="22"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
     </row>
     <row r="17" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
@@ -1584,14 +1643,14 @@
       <c r="D17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="G17" s="28"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
+      <c r="E17" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G17" s="22"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
     </row>
     <row r="18" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
@@ -1606,13 +1665,15 @@
       <c r="D18" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="H18" s="26"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K18" s="13"/>
     </row>
     <row r="19" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
@@ -1627,15 +1688,13 @@
       <c r="D19" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H19" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
+      <c r="E19" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H19" s="20"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
     </row>
     <row r="20" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
@@ -1650,42 +1709,42 @@
       <c r="D20" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H20" s="26"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-    </row>
-    <row r="21" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="2">
+      <c r="E20" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="20"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+    </row>
+    <row r="21" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="27">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="28">
         <v>7350486446</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="E21" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G21" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H21" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
+      <c r="E21" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F21" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G21" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H21" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I21" s="30"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="30"/>
     </row>
     <row r="22" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="2">
@@ -1700,15 +1759,15 @@
       <c r="D22" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E22" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H22" s="26"/>
-      <c r="I22" s="14">
+      <c r="E22" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H22" s="20"/>
+      <c r="I22" s="13">
         <v>1</v>
       </c>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
     </row>
     <row r="23" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="2">
@@ -1723,71 +1782,75 @@
       <c r="D23" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E23" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H23" s="26"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
-    </row>
-    <row r="24" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="2">
+      <c r="E23" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H23" s="20"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+    </row>
+    <row r="24" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="27">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="28">
         <v>9890737620</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G24" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H24" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-    </row>
-    <row r="25" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="2">
+      <c r="E24" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F24" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G24" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H24" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I24" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30"/>
+    </row>
+    <row r="25" spans="1:11" s="33" customFormat="1" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="27">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="28">
         <v>7499115466</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G25" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H25" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
+      <c r="E25" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F25" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G25" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H25" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I25" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J25" s="30"/>
+      <c r="K25" s="30"/>
     </row>
     <row r="26" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="2">
@@ -1802,69 +1865,75 @@
       <c r="D26" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E26" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H26" s="26"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-    </row>
-    <row r="27" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="E26" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H26" s="20"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+    </row>
+    <row r="27" spans="1:11" s="36" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="3">
         <v>7249155158</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E27" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G27" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H27" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-    </row>
-    <row r="28" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="2">
+      <c r="E27" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="G27" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H27" s="35" t="s">
+        <v>161</v>
+      </c>
+      <c r="I27" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="J27" s="34"/>
+      <c r="K27" s="34"/>
+    </row>
+    <row r="28" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="27">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="28">
         <v>7387857040</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="E28" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G28" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H28" s="26"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
+      <c r="E28" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F28" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G28" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H28" s="32"/>
+      <c r="I28" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J28" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K28" s="30"/>
     </row>
     <row r="29" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="2">
@@ -1879,74 +1948,82 @@
       <c r="D29" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E29" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="H29" s="26"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-    </row>
-    <row r="30" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="2">
+      <c r="E29" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="H29" s="20"/>
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+    </row>
+    <row r="30" spans="1:11" s="33" customFormat="1" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="27">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="28">
         <v>9503578446</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="E30" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G30" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H30" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
-    </row>
-    <row r="31" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="2">
+      <c r="E30" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F30" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G30" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H30" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I30" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J30" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K30" s="30"/>
+    </row>
+    <row r="31" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="27">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C31" s="28">
         <v>9226731346</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="E31" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G31" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H31" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
+      <c r="E31" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F31" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G31" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H31" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I31" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J31" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K31" s="30"/>
     </row>
     <row r="32" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="2">
@@ -1961,13 +2038,13 @@
       <c r="D32" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E32" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H32" s="26"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="14"/>
-      <c r="K32" s="14"/>
+      <c r="E32" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H32" s="20"/>
+      <c r="I32" s="13"/>
+      <c r="J32" s="13"/>
+      <c r="K32" s="13"/>
     </row>
     <row r="33" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="2">
@@ -1982,13 +2059,13 @@
       <c r="D33" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E33" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H33" s="26"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
+      <c r="E33" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H33" s="20"/>
+      <c r="I33" s="13"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="13"/>
     </row>
     <row r="34" spans="1:11" ht="41.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="2">
@@ -2003,46 +2080,50 @@
       <c r="D34" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E34" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F34" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G34" s="30"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="14"/>
-      <c r="K34" s="14"/>
-    </row>
-    <row r="35" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="2">
+      <c r="E34" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G34" s="24"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="13"/>
+      <c r="J34" s="13"/>
+      <c r="K34" s="13"/>
+    </row>
+    <row r="35" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="27">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="4">
+      <c r="C35" s="28">
         <v>7715045931</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="E35" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F35" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G35" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H35" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I35" s="14"/>
-      <c r="J35" s="14"/>
-      <c r="K35" s="14"/>
+      <c r="E35" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F35" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G35" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H35" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I35" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J35" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K35" s="30"/>
     </row>
     <row r="36" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="2">
@@ -2057,43 +2138,49 @@
       <c r="D36" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E36" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F36" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="H36" s="26"/>
-      <c r="I36" s="14"/>
-      <c r="J36" s="14"/>
-      <c r="K36" s="14"/>
-    </row>
-    <row r="37" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="2">
+      <c r="E36" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="H36" s="20"/>
+      <c r="I36" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="J36" s="13"/>
+      <c r="K36" s="13"/>
+    </row>
+    <row r="37" spans="1:11" s="33" customFormat="1" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="27">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="4">
+      <c r="C37" s="28">
         <v>8010613326</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="E37" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F37" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G37" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H37" s="26"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="14"/>
-      <c r="K37" s="14"/>
+      <c r="E37" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F37" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G37" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H37" s="32"/>
+      <c r="I37" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J37" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K37" s="30"/>
     </row>
     <row r="38" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="2">
@@ -2108,16 +2195,18 @@
       <c r="D38" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E38" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="G38" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H38" s="26"/>
-      <c r="I38" s="14"/>
-      <c r="J38" s="14"/>
-      <c r="K38" s="14"/>
+      <c r="E38" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G38" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="H38" s="20"/>
+      <c r="I38" s="13"/>
+      <c r="J38" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K38" s="13"/>
     </row>
     <row r="39" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="2">
@@ -2132,21 +2221,23 @@
       <c r="D39" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E39" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F39" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G39" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H39" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I39" s="14"/>
-      <c r="J39" s="14"/>
-      <c r="K39" s="14"/>
+      <c r="E39" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G39" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="H39" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I39" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="J39" s="13"/>
+      <c r="K39" s="13"/>
     </row>
     <row r="40" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="2">
@@ -2161,17 +2252,19 @@
       <c r="D40" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E40" s="11" t="s">
+      <c r="E40" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="F40" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G40" s="30"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="14"/>
-      <c r="K40" s="14"/>
+      <c r="F40" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G40" s="24"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="13"/>
+      <c r="J40" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K40" s="13"/>
     </row>
     <row r="41" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="2">
@@ -2186,13 +2279,13 @@
       <c r="D41" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E41" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="H41" s="26"/>
-      <c r="I41" s="14"/>
-      <c r="J41" s="14"/>
-      <c r="K41" s="14"/>
+      <c r="E41" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H41" s="20"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
     </row>
     <row r="42" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="2">
@@ -2207,74 +2300,78 @@
       <c r="D42" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E42" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="G42" s="30"/>
-      <c r="H42" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I42" s="14"/>
-      <c r="J42" s="14"/>
-      <c r="K42" s="14"/>
-    </row>
-    <row r="43" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="2">
+      <c r="E42" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G42" s="24"/>
+      <c r="H42" s="20"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="13"/>
+      <c r="K42" s="13"/>
+    </row>
+    <row r="43" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="27">
         <v>42</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="C43" s="3">
+      <c r="C43" s="28">
         <v>9064193565</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="E43" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F43" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G43" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H43" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I43" s="14"/>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-    </row>
-    <row r="44" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="2">
+      <c r="E43" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F43" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G43" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H43" s="32"/>
+      <c r="I43" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J43" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K43" s="30"/>
+    </row>
+    <row r="44" spans="1:11" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="27">
         <v>43</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="28">
         <v>9021750609</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="E44" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F44" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G44" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H44" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I44" s="14"/>
-      <c r="J44" s="14"/>
-      <c r="K44" s="14"/>
+      <c r="E44" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="F44" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G44" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H44" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I44" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J44" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K44" s="30"/>
     </row>
     <row r="45" spans="1:11" ht="41.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="2">
@@ -2289,19 +2386,19 @@
       <c r="D45" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E45" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F45" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G45" s="30"/>
-      <c r="H45" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I45" s="14"/>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
+      <c r="E45" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F45" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G45" s="24"/>
+      <c r="H45" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I45" s="13"/>
+      <c r="J45" s="13"/>
+      <c r="K45" s="13"/>
     </row>
     <row r="46" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="2">
@@ -2316,15 +2413,13 @@
       <c r="D46" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E46" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="H46" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I46" s="14"/>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
+      <c r="E46" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H46" s="20"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="13"/>
+      <c r="K46" s="13"/>
     </row>
     <row r="47" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="2">
@@ -2339,21 +2434,21 @@
       <c r="D47" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E47" s="10" t="s">
+      <c r="E47" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="F47" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G47" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="H47" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I47" s="14"/>
-      <c r="J47" s="14"/>
-      <c r="K47" s="14"/>
+      <c r="F47" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G47" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="H47" s="20"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K47" s="13"/>
     </row>
     <row r="48" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="2">
@@ -2368,15 +2463,15 @@
       <c r="D48" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E48" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="H48" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
+      <c r="E48" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H48" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I48" s="13"/>
+      <c r="J48" s="13"/>
+      <c r="K48" s="13"/>
     </row>
     <row r="49" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="2">
@@ -2391,16 +2486,16 @@
       <c r="D49" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E49" s="10" t="s">
+      <c r="E49" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F49" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="H49" s="26"/>
-      <c r="I49" s="14"/>
-      <c r="J49" s="14"/>
-      <c r="K49" s="14"/>
+      <c r="F49" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="H49" s="20"/>
+      <c r="I49" s="13"/>
+      <c r="J49" s="13"/>
+      <c r="K49" s="13"/>
     </row>
     <row r="50" spans="1:11" ht="41.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="2">
@@ -2415,13 +2510,13 @@
       <c r="D50" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="E50" s="10" t="s">
+      <c r="E50" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="H50" s="26"/>
-      <c r="I50" s="14"/>
-      <c r="J50" s="14"/>
-      <c r="K50" s="14"/>
+      <c r="H50" s="20"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="13"/>
+      <c r="K50" s="13"/>
     </row>
     <row r="51" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="2">
@@ -2436,16 +2531,16 @@
       <c r="D51" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E51" s="10" t="s">
+      <c r="E51" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G51" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H51" s="26"/>
-      <c r="I51" s="14"/>
-      <c r="J51" s="14"/>
-      <c r="K51" s="14"/>
+      <c r="G51" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H51" s="20"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="13"/>
+      <c r="K51" s="13"/>
     </row>
     <row r="52" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="2">
@@ -2460,13 +2555,13 @@
       <c r="D52" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E52" s="10" t="s">
+      <c r="E52" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H52" s="26"/>
-      <c r="I52" s="14"/>
-      <c r="J52" s="14"/>
-      <c r="K52" s="14"/>
+      <c r="H52" s="20"/>
+      <c r="I52" s="13"/>
+      <c r="J52" s="13"/>
+      <c r="K52" s="13"/>
     </row>
     <row r="53" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="2">
@@ -2481,13 +2576,13 @@
       <c r="D53" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E53" s="10" t="s">
+      <c r="E53" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H53" s="26"/>
-      <c r="I53" s="14"/>
-      <c r="J53" s="14"/>
-      <c r="K53" s="14"/>
+      <c r="H53" s="20"/>
+      <c r="I53" s="13"/>
+      <c r="J53" s="13"/>
+      <c r="K53" s="13"/>
     </row>
     <row r="54" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="2">
@@ -2502,13 +2597,13 @@
       <c r="D54" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="E54" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H54" s="26"/>
-      <c r="I54" s="14"/>
-      <c r="J54" s="14"/>
-      <c r="K54" s="14"/>
+      <c r="H54" s="20"/>
+      <c r="I54" s="13"/>
+      <c r="J54" s="13"/>
+      <c r="K54" s="13"/>
     </row>
     <row r="55" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="2">
@@ -2517,25 +2612,25 @@
       <c r="B55" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C55" s="6">
+      <c r="C55" s="5">
         <v>8482971951</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E55" s="10" t="s">
+      <c r="E55" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F55" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G55" s="29" t="s">
-        <v>161</v>
-      </c>
-      <c r="H55" s="26"/>
-      <c r="I55" s="14"/>
-      <c r="J55" s="14"/>
-      <c r="K55" s="14"/>
+      <c r="F55" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G55" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="H55" s="20"/>
+      <c r="I55" s="13"/>
+      <c r="J55" s="13"/>
+      <c r="K55" s="13"/>
     </row>
     <row r="56" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="2">
@@ -2550,16 +2645,16 @@
       <c r="D56" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E56" s="10" t="s">
+      <c r="E56" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G56" s="29" t="s">
-        <v>161</v>
-      </c>
-      <c r="H56" s="26"/>
-      <c r="I56" s="14"/>
-      <c r="J56" s="14"/>
-      <c r="K56" s="14"/>
+      <c r="G56" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="H56" s="20"/>
+      <c r="I56" s="13"/>
+      <c r="J56" s="13"/>
+      <c r="K56" s="13"/>
     </row>
     <row r="57" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="2">
@@ -2574,14 +2669,14 @@
       <c r="D57" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E57" s="10" t="s">
+      <c r="E57" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G57" s="28"/>
-      <c r="H57" s="26"/>
-      <c r="I57" s="14"/>
-      <c r="J57" s="14"/>
-      <c r="K57" s="14"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="20"/>
+      <c r="I57" s="13"/>
+      <c r="J57" s="13"/>
+      <c r="K57" s="13"/>
     </row>
     <row r="58" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="2">
@@ -2596,13 +2691,15 @@
       <c r="D58" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E58" s="10" t="s">
+      <c r="E58" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H58" s="26"/>
-      <c r="I58" s="14"/>
-      <c r="J58" s="14"/>
-      <c r="K58" s="14"/>
+      <c r="H58" s="20"/>
+      <c r="I58" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="J58" s="13"/>
+      <c r="K58" s="13"/>
     </row>
     <row r="59" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="2">
@@ -2617,13 +2714,13 @@
       <c r="D59" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E59" s="10" t="s">
+      <c r="E59" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H59" s="26"/>
-      <c r="I59" s="14"/>
-      <c r="J59" s="14"/>
-      <c r="K59" s="14"/>
+      <c r="H59" s="20"/>
+      <c r="I59" s="13"/>
+      <c r="J59" s="13"/>
+      <c r="K59" s="13"/>
     </row>
     <row r="60" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="2">
@@ -2632,22 +2729,22 @@
       <c r="B60" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C60" s="7">
+      <c r="C60" s="6">
         <v>8459123525</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E60" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F60" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="H60" s="26"/>
-      <c r="I60" s="14"/>
-      <c r="J60" s="14"/>
-      <c r="K60" s="14"/>
+      <c r="E60" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F60" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="H60" s="20"/>
+      <c r="I60" s="13"/>
+      <c r="J60" s="13"/>
+      <c r="K60" s="13"/>
     </row>
     <row r="61" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="2">
@@ -2656,21 +2753,23 @@
       <c r="B61" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C61" s="7">
+      <c r="C61" s="6">
         <v>8010312022</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E61" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="H61" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I61" s="14"/>
-      <c r="J61" s="14"/>
-      <c r="K61" s="14"/>
+      <c r="E61" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="H61" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I61" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="J61" s="13"/>
+      <c r="K61" s="13"/>
     </row>
     <row r="62" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="2">
@@ -2679,19 +2778,19 @@
       <c r="B62" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C62" s="7">
+      <c r="C62" s="6">
         <v>7448160689</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E62" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="H62" s="26"/>
-      <c r="I62" s="14"/>
-      <c r="J62" s="14"/>
-      <c r="K62" s="14"/>
+      <c r="E62" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="H62" s="20"/>
+      <c r="I62" s="13"/>
+      <c r="J62" s="13"/>
+      <c r="K62" s="13"/>
     </row>
     <row r="63" spans="1:11" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="2">
@@ -2700,33 +2799,31 @@
       <c r="B63" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C63" s="7">
+      <c r="C63" s="6">
         <v>9922070611</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E63" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F63" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G63" s="29" t="s">
-        <v>161</v>
-      </c>
-      <c r="H63" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I63" s="14"/>
-      <c r="J63" s="14"/>
-      <c r="K63" s="14"/>
+      <c r="E63" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F63" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G63" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="H63" s="20"/>
+      <c r="I63" s="13"/>
+      <c r="J63" s="13"/>
+      <c r="K63" s="13"/>
     </row>
     <row r="64" spans="1:11" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="2">
         <v>63</v>
       </c>
-      <c r="B64" s="8" t="s">
+      <c r="B64" s="7" t="s">
         <v>133</v>
       </c>
       <c r="C64" s="3">
@@ -2735,14 +2832,16 @@
       <c r="D64" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E64" s="10" t="s">
+      <c r="E64" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G64" s="28"/>
-      <c r="H64" s="26"/>
-      <c r="I64" s="14"/>
-      <c r="J64" s="14"/>
-      <c r="K64" s="14"/>
+      <c r="G64" s="22"/>
+      <c r="H64" s="20"/>
+      <c r="I64" s="13"/>
+      <c r="J64" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K64" s="13"/>
     </row>
     <row r="65" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="2">
@@ -2757,13 +2856,13 @@
       <c r="D65" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E65" s="10" t="s">
+      <c r="E65" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H65" s="26"/>
-      <c r="I65" s="14"/>
-      <c r="J65" s="14"/>
-      <c r="K65" s="14"/>
+      <c r="H65" s="20"/>
+      <c r="I65" s="13"/>
+      <c r="J65" s="13"/>
+      <c r="K65" s="13"/>
     </row>
     <row r="66" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="2">
@@ -2778,19 +2877,19 @@
       <c r="D66" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="E66" s="10" t="s">
+      <c r="E66" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H66" s="26"/>
-      <c r="I66" s="14"/>
-      <c r="J66" s="14"/>
-      <c r="K66" s="14"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="13"/>
+      <c r="J66" s="13"/>
+      <c r="K66" s="13"/>
     </row>
     <row r="67" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="2">
         <v>66</v>
       </c>
-      <c r="B67" s="8" t="s">
+      <c r="B67" s="7" t="s">
         <v>139</v>
       </c>
       <c r="C67" s="3">
@@ -2799,16 +2898,18 @@
       <c r="D67" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="E67" s="10" t="s">
+      <c r="E67" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G67" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H67" s="26"/>
-      <c r="I67" s="14"/>
-      <c r="J67" s="14"/>
-      <c r="K67" s="14"/>
+      <c r="G67" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H67" s="20"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K67" s="13"/>
     </row>
     <row r="68" spans="1:12" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="2">
@@ -2823,106 +2924,118 @@
       <c r="D68" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="E68" s="10" t="s">
+      <c r="E68" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H68" s="26"/>
-      <c r="I68" s="14"/>
-      <c r="J68" s="14"/>
-      <c r="K68" s="14"/>
-    </row>
-    <row r="69" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A69" s="2">
+      <c r="H68" s="20"/>
+      <c r="I68" s="13"/>
+      <c r="J68" s="13"/>
+      <c r="K68" s="13"/>
+    </row>
+    <row r="69" spans="1:12" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A69" s="27">
         <v>68</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="B69" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="C69" s="3">
+      <c r="C69" s="28">
         <v>8451042496</v>
       </c>
-      <c r="D69" s="3" t="s">
+      <c r="D69" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="E69" s="10" t="s">
+      <c r="E69" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="F69" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G69" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H69" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I69" s="14"/>
-      <c r="J69" s="14"/>
-      <c r="K69" s="14"/>
-    </row>
-    <row r="70" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A70" s="2">
+      <c r="F69" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G69" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H69" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I69" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J69" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K69" s="30"/>
+    </row>
+    <row r="70" spans="1:12" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A70" s="27">
         <v>69</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="B70" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C70" s="3">
+      <c r="C70" s="28">
         <v>7666361933</v>
       </c>
-      <c r="D70" s="3" t="s">
+      <c r="D70" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="E70" s="10" t="s">
+      <c r="E70" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="F70" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G70" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H70" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I70" s="14"/>
-      <c r="J70" s="14"/>
-      <c r="K70" s="14"/>
-    </row>
-    <row r="71" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A71" s="2">
+      <c r="F70" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G70" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H70" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I70" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J70" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K70" s="30"/>
+    </row>
+    <row r="71" spans="1:12" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A71" s="27">
         <v>70</v>
       </c>
-      <c r="B71" s="8" t="s">
+      <c r="B71" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="C71" s="8">
+      <c r="C71" s="28">
         <v>7820816633</v>
       </c>
-      <c r="D71" s="3" t="s">
+      <c r="D71" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="E71" s="10" t="s">
+      <c r="E71" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="F71" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G71" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H71" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I71" s="14"/>
-      <c r="J71" s="14"/>
-      <c r="K71" s="14"/>
+      <c r="F71" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G71" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H71" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I71" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J71" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K71" s="30"/>
     </row>
     <row r="72" spans="1:12" ht="68.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="2">
         <v>71</v>
       </c>
-      <c r="B72" s="8" t="s">
+      <c r="B72" s="7" t="s">
         <v>149</v>
       </c>
       <c r="C72" s="3">
@@ -2931,56 +3044,62 @@
       <c r="D72" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="E72" s="10" t="s">
+      <c r="E72" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F72" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G72" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H72" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I72" s="14"/>
-      <c r="J72" s="14"/>
-      <c r="K72" s="14"/>
-    </row>
-    <row r="73" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A73" s="2">
+      <c r="F72" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="G72" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H72" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I72" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="J72" s="13"/>
+      <c r="K72" s="13"/>
+    </row>
+    <row r="73" spans="1:12" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A73" s="27">
         <v>72</v>
       </c>
-      <c r="B73" s="8" t="s">
+      <c r="B73" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="C73" s="3">
+      <c r="C73" s="28">
         <v>8767152381</v>
       </c>
-      <c r="D73" s="3" t="s">
+      <c r="D73" s="28" t="s">
         <v>152</v>
       </c>
-      <c r="E73" s="10" t="s">
+      <c r="E73" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="F73" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G73" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H73" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I73" s="14"/>
-      <c r="J73" s="14"/>
-      <c r="K73" s="14"/>
+      <c r="F73" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G73" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H73" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I73" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J73" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="K73" s="30"/>
     </row>
     <row r="74" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="2">
         <v>73</v>
       </c>
-      <c r="B74" s="8" t="s">
+      <c r="B74" s="7" t="s">
         <v>153</v>
       </c>
       <c r="C74" s="3">
@@ -2989,19 +3108,19 @@
       <c r="D74" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="E74" s="10" t="s">
+      <c r="E74" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="H74" s="26"/>
-      <c r="I74" s="14"/>
-      <c r="J74" s="14"/>
-      <c r="K74" s="14"/>
+      <c r="H74" s="20"/>
+      <c r="I74" s="13"/>
+      <c r="J74" s="13"/>
+      <c r="K74" s="13"/>
     </row>
     <row r="75" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="2">
         <v>74</v>
       </c>
-      <c r="B75" s="8" t="s">
+      <c r="B75" s="7" t="s">
         <v>155</v>
       </c>
       <c r="C75" s="3">
@@ -3010,90 +3129,96 @@
       <c r="D75" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="E75" s="10" t="s">
+      <c r="E75" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H75" s="26"/>
-      <c r="I75" s="14"/>
-      <c r="J75" s="14"/>
-      <c r="K75" s="14"/>
-    </row>
-    <row r="76" spans="1:12" ht="55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A76" s="2">
+      <c r="H75" s="20"/>
+      <c r="I75" s="13"/>
+      <c r="J75" s="13"/>
+      <c r="K75" s="13"/>
+    </row>
+    <row r="76" spans="1:12" s="33" customFormat="1" ht="55" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A76" s="27">
         <v>75</v>
       </c>
-      <c r="B76" s="8" t="s">
+      <c r="B76" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="C76" s="5"/>
-      <c r="D76" s="8" t="s">
+      <c r="C76" s="41"/>
+      <c r="D76" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="E76" s="10" t="s">
+      <c r="E76" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="F76" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="G76" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="H76" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I76" s="14"/>
-      <c r="J76" s="14"/>
-      <c r="K76" s="14"/>
-    </row>
-    <row r="77" spans="1:12" ht="68" x14ac:dyDescent="0.35">
-      <c r="A77" s="15">
+      <c r="F76" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G76" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="H76" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I76" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J76" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="K76" s="30"/>
+    </row>
+    <row r="77" spans="1:12" s="33" customFormat="1" ht="68" x14ac:dyDescent="0.35">
+      <c r="A77" s="37">
         <v>76</v>
       </c>
-      <c r="B77" s="16" t="s">
+      <c r="B77" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="C77" s="17">
+      <c r="C77" s="38">
         <v>8237450604</v>
       </c>
-      <c r="D77" s="17" t="s">
+      <c r="D77" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="E77" s="18" t="s">
+      <c r="E77" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="F77" s="19"/>
-      <c r="G77" s="28"/>
-      <c r="H77" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="I77" s="14"/>
-      <c r="J77" s="14"/>
-      <c r="K77" s="14"/>
-    </row>
-    <row r="78" spans="1:12" s="14" customFormat="1" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="14">
+      <c r="F77" s="40"/>
+      <c r="G77" s="31"/>
+      <c r="H77" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="I77" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J77" s="30"/>
+      <c r="K77" s="30"/>
+    </row>
+    <row r="78" spans="1:12" s="13" customFormat="1" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A78" s="13">
         <v>77</v>
       </c>
-      <c r="B78" s="21" t="s">
+      <c r="B78" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="G78" s="29"/>
-      <c r="H78" s="26"/>
-      <c r="L78" s="22"/>
-    </row>
-    <row r="79" spans="1:12" s="14" customFormat="1" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="23">
+      <c r="G78" s="23"/>
+      <c r="H78" s="20"/>
+      <c r="L78" s="16"/>
+    </row>
+    <row r="79" spans="1:12" s="13" customFormat="1" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="17">
         <v>78</v>
       </c>
-      <c r="B79" s="21" t="s">
+      <c r="B79" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="G79" s="29"/>
-      <c r="H79" s="26"/>
+      <c r="G79" s="23"/>
+      <c r="H79" s="20"/>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="F80" s="20"/>
-      <c r="G80" s="31"/>
+      <c r="F80" s="14"/>
+      <c r="G80" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>